<commit_message>
mAP calc for all models
</commit_message>
<xml_diff>
--- a/mAP_results.xlsx
+++ b/mAP_results.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,7 +497,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Class-agnostic mAP 50:95</t>
+          <t>CA mAP 50:95</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CA mAP 50</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CA mAP 75</t>
         </is>
       </c>
     </row>
@@ -525,16 +535,22 @@
         <v>0.6527804375799173</v>
       </c>
       <c r="G2" t="n">
+        <v>0.1178996984685442</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.2624451808019757</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.2548315577088544</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.2381503153945095</v>
+        <v>0.067044879724661</v>
       </c>
       <c r="J2" t="n">
+        <v>0.3191331629176098</v>
+      </c>
+      <c r="K2" t="n">
         <v>0.6877148883005395</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.205714316891391</v>
       </c>
     </row>
     <row r="3">
@@ -561,16 +577,22 @@
         <v>0.5019818393705298</v>
       </c>
       <c r="G3" t="n">
+        <v>0.064131804101156</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.1692502344034677</v>
       </c>
-      <c r="H3" t="n">
-        <v>0.1556167948855464</v>
-      </c>
       <c r="I3" t="n">
-        <v>0.1340903427641949</v>
+        <v>0.0240128504426048</v>
       </c>
       <c r="J3" t="n">
+        <v>0.1928083991687326</v>
+      </c>
+      <c r="K3" t="n">
         <v>0.5236704034080688</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0666622862770173</v>
       </c>
     </row>
     <row r="4">
@@ -589,16 +611,22 @@
         <v>0.5041561785604179</v>
       </c>
       <c r="G4" t="n">
+        <v>0.0643930790791719</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.1695812035650267</v>
       </c>
-      <c r="H4" t="n">
-        <v>0.1552394699410264</v>
-      </c>
       <c r="I4" t="n">
-        <v>0.1353826658843398</v>
+        <v>0.0243523161270855</v>
       </c>
       <c r="J4" t="n">
+        <v>0.1937377912653786</v>
+      </c>
+      <c r="K4" t="n">
         <v>0.5258766426107448</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0685008904692356</v>
       </c>
     </row>
     <row r="5">
@@ -625,16 +653,22 @@
         <v>0.5317640696353413</v>
       </c>
       <c r="G5" t="n">
+        <v>0.1320526781432406</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.3674855316077661</v>
       </c>
-      <c r="H5" t="n">
-        <v>0.3092826990990522</v>
-      </c>
       <c r="I5" t="n">
-        <v>0.2419732364480355</v>
+        <v>0.0595172966936393</v>
       </c>
       <c r="J5" t="n">
+        <v>0.2206520764239244</v>
+      </c>
+      <c r="K5" t="n">
         <v>0.5847548914246699</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.1259433298253978</v>
       </c>
     </row>
     <row r="6">
@@ -653,16 +687,22 @@
         <v>0.5450784940821434</v>
       </c>
       <c r="G6" t="n">
+        <v>0.1350256182042557</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.3752494376668481</v>
       </c>
-      <c r="H6" t="n">
-        <v>0.3123707901940489</v>
-      </c>
       <c r="I6" t="n">
-        <v>0.2459884481853903</v>
+        <v>0.06272455481036079</v>
       </c>
       <c r="J6" t="n">
+        <v>0.2254931211971026</v>
+      </c>
+      <c r="K6" t="n">
         <v>0.5992544885460649</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1330026792430242</v>
       </c>
     </row>
     <row r="7">
@@ -689,16 +729,22 @@
         <v>0.7198529599552497</v>
       </c>
       <c r="G7" t="n">
+        <v>0.189585593381839</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.3381634192657484</v>
       </c>
-      <c r="H7" t="n">
-        <v>0.3339539635767536</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.3294712574319242</v>
+        <v>0.1670289712549293</v>
       </c>
       <c r="J7" t="n">
+        <v>0.4298705763438617</v>
+      </c>
+      <c r="K7" t="n">
         <v>0.7531869175377615</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.446126204190736</v>
       </c>
     </row>
     <row r="8">
@@ -725,16 +771,22 @@
         <v>0.4242485069770008</v>
       </c>
       <c r="G8" t="n">
+        <v>0.0617604603127956</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.1433716956188824</v>
       </c>
-      <c r="H8" t="n">
-        <v>0.1353261573489375</v>
-      </c>
       <c r="I8" t="n">
-        <v>0.1176644002619575</v>
+        <v>0.0378495780002211</v>
       </c>
       <c r="J8" t="n">
+        <v>0.2091315125480065</v>
+      </c>
+      <c r="K8" t="n">
         <v>0.4901044190577212</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.1307535843688784</v>
       </c>
     </row>
     <row r="9">
@@ -753,16 +805,22 @@
         <v>0.4392775149849883</v>
       </c>
       <c r="G9" t="n">
+        <v>0.0623079958416592</v>
+      </c>
+      <c r="H9" t="n">
         <v>0.1487279634121421</v>
       </c>
-      <c r="H9" t="n">
-        <v>0.1379302541309899</v>
-      </c>
       <c r="I9" t="n">
-        <v>0.1188396992066528</v>
+        <v>0.0372189917417575</v>
       </c>
       <c r="J9" t="n">
+        <v>0.2084649037996507</v>
+      </c>
+      <c r="K9" t="n">
         <v>0.5029997652590329</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.1248484063255638</v>
       </c>
     </row>
     <row r="10">
@@ -781,16 +839,22 @@
         <v>0.422511753800949</v>
       </c>
       <c r="G10" t="n">
+        <v>0.0619248272143439</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.1431357454364108</v>
       </c>
-      <c r="H10" t="n">
-        <v>0.1326950312345982</v>
-      </c>
       <c r="I10" t="n">
-        <v>0.1148081514781631</v>
+        <v>0.0396016420889505</v>
       </c>
       <c r="J10" t="n">
+        <v>0.2109041457581544</v>
+      </c>
+      <c r="K10" t="n">
         <v>0.4938002433354184</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.1335044511127464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add weighted mAP code and yolo mAP pipeline for Rishabh
</commit_message>
<xml_diff>
--- a/mAP_results.xlsx
+++ b/mAP_results.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,32 +482,37 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>mAP 50:95</t>
+          <t>Weighted mAP@50</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>mAP 50</t>
+          <t>mAP@50:95</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>mAP 75</t>
+          <t>mAP@50</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>CA mAP 50:95</t>
+          <t>mAP@75</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>CA mAP 50</t>
+          <t>CA mAP@50:95</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>CA mAP 75</t>
+          <t>CA mAP@50</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CA mAP@75</t>
         </is>
       </c>
     </row>
@@ -526,31 +531,34 @@
         <v>36</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1221122112211221</v>
+        <v>0.122112</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0124428936048877</v>
+        <v>0.012443</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6527804375799173</v>
+        <v>0.65278</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1178996984685442</v>
+        <v>0.580084</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2624451808019757</v>
+        <v>0.1179</v>
       </c>
       <c r="I2" t="n">
-        <v>0.067044879724661</v>
+        <v>0.262445</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3191331629176098</v>
+        <v>0.06704499999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6877148883005395</v>
+        <v>0.319133</v>
       </c>
       <c r="L2" t="n">
-        <v>0.205714316891391</v>
+        <v>0.687715</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.205714</v>
       </c>
     </row>
     <row r="3">
@@ -571,28 +579,31 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0057688638398735</v>
+        <v>0.005769</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5019818393705298</v>
+        <v>0.501982</v>
       </c>
       <c r="G3" t="n">
-        <v>0.064131804101156</v>
+        <v>0.444844</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1692502344034677</v>
+        <v>0.06413199999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0240128504426048</v>
+        <v>0.16925</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1928083991687326</v>
+        <v>0.024013</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5236704034080688</v>
+        <v>0.192808</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0666622862770173</v>
+        <v>0.52367</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.066662</v>
       </c>
     </row>
     <row r="4">
@@ -605,28 +616,31 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0045874321346622</v>
+        <v>0.004587</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5041561785604179</v>
+        <v>0.504156</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0643930790791719</v>
+        <v>0.446643</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1695812035650267</v>
+        <v>0.06439300000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0243523161270855</v>
+        <v>0.169581</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1937377912653786</v>
+        <v>0.024352</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5258766426107448</v>
+        <v>0.193738</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0685008904692356</v>
+        <v>0.525877</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.06850100000000001</v>
       </c>
     </row>
     <row r="5">
@@ -644,31 +658,34 @@
         <v>50</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2178217821782178</v>
+        <v>0.217822</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3528707430097394</v>
+        <v>0.352871</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5317640696353413</v>
+        <v>0.531764</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1320526781432406</v>
+        <v>0.469825</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3674855316077661</v>
+        <v>0.132053</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0595172966936393</v>
+        <v>0.367486</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2206520764239244</v>
+        <v>0.059517</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5847548914246699</v>
+        <v>0.220652</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1259433298253978</v>
+        <v>0.584755</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.125943</v>
       </c>
     </row>
     <row r="6">
@@ -678,31 +695,34 @@
         <v>45</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2178217821782178</v>
+        <v>0.217822</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3628480367401833</v>
+        <v>0.362848</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5450784940821434</v>
+        <v>0.545078</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1350256182042557</v>
+        <v>0.481592</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3752494376668481</v>
+        <v>0.135026</v>
       </c>
       <c r="I6" t="n">
-        <v>0.06272455481036079</v>
+        <v>0.375249</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2254931211971026</v>
+        <v>0.062725</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5992544885460649</v>
+        <v>0.225493</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1330026792430242</v>
+        <v>0.599254</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.133003</v>
       </c>
     </row>
     <row r="7">
@@ -720,31 +740,34 @@
         <v>50</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2244224422442244</v>
+        <v>0.224422</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0702148555977712</v>
+        <v>0.070215</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7198529599552497</v>
+        <v>0.719853</v>
       </c>
       <c r="G7" t="n">
-        <v>0.189585593381839</v>
+        <v>0.646481</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3381634192657484</v>
+        <v>0.189586</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1670289712549293</v>
+        <v>0.338163</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4298705763438617</v>
+        <v>0.167029</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7531869175377615</v>
+        <v>0.429871</v>
       </c>
       <c r="L7" t="n">
-        <v>0.446126204190736</v>
+        <v>0.7531870000000001</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.446126</v>
       </c>
     </row>
     <row r="8">
@@ -765,28 +788,31 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0058665798796465</v>
+        <v>0.005867</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4242485069770008</v>
+        <v>0.424249</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0617604603127956</v>
+        <v>0.376064</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1433716956188824</v>
+        <v>0.06176</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0378495780002211</v>
+        <v>0.143372</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2091315125480065</v>
+        <v>0.03785</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4901044190577212</v>
+        <v>0.209132</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1307535843688784</v>
+        <v>0.490104</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.130754</v>
       </c>
     </row>
     <row r="9">
@@ -799,28 +825,31 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0069063752514379</v>
+        <v>0.006906</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4392775149849883</v>
+        <v>0.439278</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0623079958416592</v>
+        <v>0.389475</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1487279634121421</v>
+        <v>0.062308</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0372189917417575</v>
+        <v>0.148728</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2084649037996507</v>
+        <v>0.037219</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5029997652590329</v>
+        <v>0.208465</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1248484063255638</v>
+        <v>0.503</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.124848</v>
       </c>
     </row>
     <row r="10">
@@ -833,28 +862,31 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0068954825082836</v>
+        <v>0.006895</v>
       </c>
       <c r="F10" t="n">
-        <v>0.422511753800949</v>
+        <v>0.422512</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0619248272143439</v>
+        <v>0.374636</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1431357454364108</v>
+        <v>0.061925</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0396016420889505</v>
+        <v>0.143136</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2109041457581544</v>
+        <v>0.039602</v>
       </c>
       <c r="K10" t="n">
-        <v>0.4938002433354184</v>
+        <v>0.210904</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1335044511127464</v>
+        <v>0.4938</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.133504</v>
       </c>
     </row>
   </sheetData>

</xml_diff>